<commit_message>
feat: add AVdb actor sync and actor db static validation
- sync_from_avdb: merge actor-mapping.xml into actor_database.xlsx
  (jsdelivr/github/url/file sources, local-first fill, tmdbid conflict merge)
- scripts/check_actor_db.py: static validation for factory xlsx
  (jp dup, keyword dup/bad commas, empty names, tmdbid dup, birth date format)
- hook check_actor_db into uv run check
- fix keyword dup in factory xlsx and extend headers to 9 columns
Co-authored-by: monkeycode-ai <monkeycode-ai@chaitin.com>
</commit_message>
<xml_diff>
--- a/resources/userdata/actor_database.xlsx
+++ b/resources/userdata/actor_database.xlsx
@@ -1123,7 +1123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col width="14" customWidth="1" style="1" min="1" max="1"/>
@@ -1172,6 +1172,16 @@
           <t>tmdb url</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>出生日期</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>简介</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -2360,7 +2370,7 @@
       </c>
       <c r="D37" s="8" t="inlineStr">
         <is>
-          <t>小野夕子,葵,Yûko Ono,Aoi Tanabo,Yuuko Ono,Satomi Nagase,おのゆうこ,あおい,AOI,Aoi,Yuko Oko,Oko Yuko</t>
+          <t>小野夕子,葵,Yûko Ono,Aoi Tanabo,Yuuko Ono,Satomi Nagase,おのゆうこ,あおい,AOI,Yuko Oko,Oko Yuko</t>
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr">

</xml_diff>